<commit_message>
Update Week 4: Modify ETL diagrams and add ETL schema image
</commit_message>
<xml_diff>
--- a/DEAI/WEEK 6/MachineLearning.xlsx
+++ b/DEAI/WEEK 6/MachineLearning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kyran\Desktop\Semester 4 Projects VSC\Roody repo\HHS-Pyhthon-Pipeline\DEAI\WEEK 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D879BB6-2465-4E11-9D9D-6215783146E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0024F2D4-7773-4381-AAA6-869D44BF32CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="18">
   <si>
     <t>Gekozen features:</t>
   </si>
@@ -73,6 +73,12 @@
   </si>
   <si>
     <t>0.6721886124684764</t>
+  </si>
+  <si>
+    <t>max_iter= 4000, eta0=0.00005</t>
+  </si>
+  <si>
+    <t>0.6718840352990239</t>
   </si>
 </sst>
 </file>
@@ -126,6 +132,143 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>251461</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>53817</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Afbeelding 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E252566-509A-A57D-B52C-CB0DF106E334}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4130041" y="7620"/>
+          <a:ext cx="2850356" cy="2171700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>213360</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>137696</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>344805</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Afbeelding 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DF59B3C-1D58-4F46-6F1A-B9F0E3A0D94C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4091940" y="2332256"/>
+          <a:ext cx="3179445" cy="2300704"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>20175</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>128589</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Afbeelding 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDA982B6-5A25-ED26-19D1-7409B04FBAD4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4030980" y="4775055"/>
+          <a:ext cx="3276600" cy="2485854"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -391,7 +534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
@@ -493,7 +636,56 @@
         <v>15</v>
       </c>
     </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="1">
+        <v>2.52075636627093E+16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="1">
+        <v>3.37733660872856E+16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add DEAI Week 7 Classificatie notebooks and resources
</commit_message>
<xml_diff>
--- a/DEAI/WEEK 6/MachineLearning.xlsx
+++ b/DEAI/WEEK 6/MachineLearning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kyran\Desktop\Semester 4 Projects VSC\Roody repo\HHS-Pyhthon-Pipeline\DEAI\WEEK 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0024F2D4-7773-4381-AAA6-869D44BF32CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE9D2AF-BDB2-4327-A076-EDD31907A92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -227,22 +227,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
+      <xdr:colOff>144781</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>20175</xdr:rowOff>
+      <xdr:rowOff>7621</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
+      <xdr:colOff>441403</xdr:colOff>
       <xdr:row>39</xdr:row>
-      <xdr:rowOff>128589</xdr:rowOff>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Afbeelding 4">
+        <xdr:cNvPr id="6" name="Afbeelding 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDA982B6-5A25-ED26-19D1-7409B04FBAD4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57CF2259-7F0D-343B-A343-A9EDC3E76D15}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -258,8 +258,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4030980" y="4775055"/>
-          <a:ext cx="3276600" cy="2485854"/>
+          <a:off x="4023361" y="4762501"/>
+          <a:ext cx="3344622" cy="2537459"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>